<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.001-01 Le bol de fraises
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.001-01.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.001-01.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin, fraisiers, plaid sous le cerisier</t>
+          <t>jardin, fraisiers, plaid sous le cerisier, bol émaillé</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorino, Nina, maman</t>
+          <t>Victorino, Nina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino veut un bol de fraises pour le goûter. Nina est plus grande, lui plus petit. Ils cueillent ensemble, haut et bas. Le bol se remplit sur le plaid.</t>
+          <t>L'eau glisse. Le bol émaillé est froid. Sur le bord, un éclat d'émail brille. Victorino veut des fraises, maintenant, avec Nina. Il lève trop haut : le bol penche, l'éclat saute. Il refuse de foncer, cueille bas, Nina haut. Merci vécu. Vers le plaid, il porte trop haut : ça roule. Il tient le fond, Nina le bord. L'éclat d'émail tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le bol émaillé est froid. Maman l'a rincé. Une goutte coule sur le bord. Les fraisiers sentent la terre. La terre est tiède. Une abeille passe, tout loin. Tu as vu la goutte ? Oui, maman. Elle brille. Oui. Je veux des fraises. Pour le goûter, sur le plaid ? Oui. En ce moment, Victorino se baisse. Les feuilles lui touchent les mains. Elles sont un peu râpeuses. Nina arrive avec un panier. Nina est plus grande. Victorino est plus petit. Ils ont des tailles différentes. Tu viens ? Oui. Ils vont près des fraisiers. Une fraise rouge est trop haut. Victorino lève la main. Il n'arrive pas. Elle est trop haut. Il y en a en bas aussi. Nina cueille la haute. Victorino cueille une basse. La basse sent le sucre. Elle est chaude ! Le soleil l'a chauffée. Vous jouez ensemble. On peut jouer ensemble. Le bol sonne un peu. Deux fraises roulent dedans. Encore une ? Oui. Une feuille colle au poignet. Victorino la retire, tout doux. La terre reste sur ses genoux. Elle est chaude, un peu sèche. On laisse l'abeille ? Oui. Tu as de la terre aux genoux. C'est le jardin.</t>
+          <t>L'eau glisse sur le bord. Elle est froide. Le bol émaillé vient du robinet. Maman l'a rincé. Papa tient le torchon bleu. Il est froid, papa ! Tu as senti l'eau ? Oui, papa. Le jardin sent la terre. La terre est tiède. Le cerisier fait de l'ombre. Un plaid attend dessous. Le plaid est prêt ? Oui, maman. Sur le bord, un éclat d'émail brille. Il est blanc, maman. Tu le vois sur le bol ? Oui, il brille. C'est l'émail, sous la lumière. Je veux des fraises. Maintenant ! Pour le goûter, sur le plaid ? Oui. Les fraisiers sentent le sucre. Les feuilles sont un peu râpeuses. Une fraise basse est chaude. Le soleil l'a chauffée. Elle est rouge, celle-là ? Oui, toute rouge. Nina arrive près du cerisier. Ses mains touchent les hautes feuilles. Tu viens ? Oui. Ils posent le bol dans l'herbe. Nina cueille une fraise haute. Elle la laisse tomber dans le bol. Le bol sonne un petit ding. Ding ! En ce moment, Victorino lève la main. Une fraise rouge est trop haut. Sa main n'arrive pas. Elle est trop haut ! Il saisit le bol trop vite. Le bol penche vers l'herbe. L'éclat d'émail saute près du bol. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas ! Papa s'accroupit à la même hauteur. Tes doigts sont près du bol ? Oui, papa. On essuie tes genoux. Voilà. C'est tiède. C'est la terre, Victorino. Une feuille colle au poignet. Victorino la retire. Nina reste près des hautes feuilles. Elle ne dit rien. La haute, Nina ! Victorino veut la haute, tout de suite. Il tend le bras trop loin.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le bol émaillé est froid. Maman l'a rincé. Une goutte coule sur le bord. Les fraisiers sentent la terre. La terre est tiède. Une abeille passe, tout loin. Tu as vu la goutte ? Oui, maman. Elle brille. Oui. Je veux des fraises. Pour le goûter, sur le plaid ? Oui. En ce moment, Victorino se baisse. Les feuilles lui touchent les mains. Elles sont un peu râpeuses. Nina arrive avec un panier. Nina est plus grande. Victorino est plus petit. Ils ont des tailles différentes. Tu viens ? Oui. Ils vont près des fraisiers. Une fraise rouge est trop haut. Victorino lève la main. Il n'arrive pas. Elle est trop haut. Il y en a en bas aussi. Nina cueille la haute. Victorino cueille une basse. La basse sent le sucre. Elle est chaude ! Le soleil l'a chauffée. Vous jouez ensemble. On peut jouer ensemble. Le bol sonne un peu. Deux fraises roulent dedans. Encore une ? Oui. Une feuille colle au poignet. Victorino la retire, tout doux. La terre reste sur ses genoux. Elle est chaude, un peu sèche. On laisse l'abeille ? Oui. Tu as de la terre aux genoux. C'est le jardin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'eau glisse sur le bord. Elle est froide. Le bol émaillé vient du robinet. Maman l'a rincé. Papa tient le torchon bleu. Il est froid, papa ! Tu as senti l'eau ? Oui, papa. Le jardin sent la terre. La terre est tiède. Le cerisier fait de l'ombre. Un plaid attend dessous. Le plaid est prêt ? Oui, maman. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat d'émail&lt;/emphasis&gt; brille. Il est blanc, maman. Tu le vois sur le bol ? Oui, il brille. C'est l'émail, sous la lumière. Je veux des fraises. Maintenant ! Pour le goûter, sur le plaid ? Oui. Les fraisiers sentent le sucre. Les feuilles sont un peu râpeuses. Une fraise basse est chaude. Le soleil l'a chauffée. Elle est rouge, celle-là ? Oui, toute rouge. Nina arrive près du cerisier. Ses mains touchent les hautes feuilles. Tu viens ? Oui. Ils posent le bol dans l'herbe. Nina cueille une fraise haute. Elle la laisse tomber dans le bol. Le bol sonne un petit ding. Ding ! En ce moment, Victorino lève la main. Une fraise rouge est trop haut. Sa main n'arrive pas. Elle est trop haut ! Il saisit le bol trop vite. Le bol penche vers l'herbe. L'éclat d'émail saute près du bol. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas ! Papa s'accroupit à la même hauteur. Tes doigts sont près du bol ? Oui, papa. On essuie tes genoux. Voilà. C'est tiède. C'est la terre, Victorino. Une feuille colle au poignet. Victorino la retire. Nina reste près des hautes feuilles. Elle ne dit rien. La haute, Nina ! Victorino veut la haute, tout de suite. Il tend le bras trop loin.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est l'après-midi. Le soleil est doux. Nora est dans le jardin. Maman est là, près des fleurs. Hugo arrive avec un seau. Hugo est plus grand que Nora. Nora est plus petite que Hugo. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Maman sourit. Nora veut du sable. Elle prend une petite pelle. Elle va vers Hugo. Elle l'invite. Nora dit : viens jouer. Hugo dit : oui. Ils jouent ensemble près du bac. Hugo porte un gros seau. Nora porte un petit seau. Les tailles différentes restent là. Les deux enfants remplissent le bac. Maman dit : vous jouez ensemble. Nora donne une pelle à Hugo. Hugo donne un moule à Nora. Ils font un gâteau de sable. Nora met un caillou dessus. Hugo met une feuille verte. Ils tapent des mains. Hugo veut la corde à sauter. La corde est un peu haute. Hugo baisse la corde. Nora tient un bout. Hugo tient l'autre bout. Ils sautent un peu. Puis ils sautent ensemble. Maman dit : encore. On invite. On joue ensemble. Petit ou grand, on joue ensemble. Nora verse de l'eau. Hugo lisse le sable. Le gâteau tient debout. Maman dit : bravo. Vous avez des tailles différentes. Et vous jouez ensemble.&lt;/slow&gt; [pause]</t>
+          <t>L'eau glisse sur le bord. Elle est froide. Le bol émaillé vient du robinet. Maman l'a rincé. Papa tient le torchon bleu. Il est froid, papa ! Tu as senti l'eau ? Oui, papa. Le jardin sent la terre. La terre est tiède. Le cerisier fait de l'ombre. Un plaid attend dessous. Le plaid est prêt ? Oui, maman. Sur le bord, un &lt;emphasis&gt;éclat d'émail&lt;/emphasis&gt; brille. Il est blanc, maman. Tu le vois sur le bol ? Oui, il brille. C'est l'émail, sous la lumière. Je veux des fraises. Maintenant ! Pour le goûter, sur le plaid ? Oui. Les fraisiers sentent le sucre. Les feuilles sont un peu râpeuses. Une fraise basse est chaude. Le soleil l'a chauffée. Elle est rouge, celle-là ? Oui, toute rouge. Nina arrive près du cerisier. Ses mains touchent les hautes feuilles. Tu viens ? Oui. Ils posent le bol dans l'herbe. Nina cueille une fraise haute. Elle la laisse tomber dans le bol. Le bol sonne un petit ding. Ding ! En ce moment, Victorino lève la main. Une fraise rouge est trop haut. Sa main n'arrive pas. Elle est trop haut ! Il saisit le bol trop vite. Le bol penche vers l'herbe. L'éclat d'émail saute près du bol. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ça ne veut pas ! Papa s'accroupit à la même hauteur. Tes doigts sont près du bol ? Oui, papa. On essuie tes genoux. Voilà. C'est tiède. C'est la terre, Victorino. Une feuille colle au poignet. Victorino la retire. Nina reste près des hautes feuilles. Elle ne dit rien. La haute, Nina ! Victorino veut la haute, tout de suite. Il tend le bras trop loin. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,18 +1246,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>éclat d'émail</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1324,58 +1324,84 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_les_fraises_maintenant_avec_nina; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le bol émaillé est froid.
+          <t>narrateur|L'eau glisse sur le bord.
+narrateur|Elle est froide.
+narrateur|Le bol émaillé vient du robinet.
 narrateur|Maman l'a rincé.
-narrateur|Une goutte coule sur le bord.
-narrateur|Les fraisiers sentent la terre.
+narrateur|Papa tient le torchon bleu.
+enfant-m|Il est froid, papa !
+papa|Tu as senti l'eau ?
+enfant-m|Oui, papa.
+narrateur|Le jardin sent la terre.
 narrateur|La terre est tiède.
-narrateur|Une abeille passe, tout loin.
-maman|Tu as vu la goutte ?
+narrateur|Le cerisier fait de l'ombre.
+narrateur|Un plaid attend dessous.
+maman|Le plaid est prêt ?
 enfant-m|Oui, maman.
-enfant-m|Elle brille.
-maman|Oui.
+narrateur|Sur le bord, un éclat d'émail brille.
+enfant-m|Il est blanc, maman.
+maman|Tu le vois sur le bol ?
+enfant-m|Oui, il brille.
+papa|C'est l'émail, sous la lumière.
 enfant-m|Je veux des fraises.
+enfant-m|Maintenant !
 maman|Pour le goûter, sur le plaid ?
 enfant-m|Oui.
-narrateur|En ce moment, Victorino se baisse.
-narrateur|Les feuilles lui touchent les mains.
-narrateur|Elles sont un peu râpeuses.
-narrateur|Nina arrive avec un panier.
-narrateur|Nina est plus grande.
-narrateur|Victorino est plus petit.
-narrateur|Ils ont des tailles différentes.
+narrateur|Les fraisiers sentent le sucre.
+narrateur|Les feuilles sont un peu râpeuses.
+narrateur|Une fraise basse est chaude.
+enfant-m|Le soleil l'a chauffée.
+papa|Elle est rouge, celle-là ?
+enfant-m|Oui, toute rouge.
+narrateur|Nina arrive près du cerisier.
+narrateur|Ses mains touchent les hautes feuilles.
 enfant-m|Tu viens ?
 copine|Oui.
-narrateur|Ils vont près des fraisiers.
+narrateur|Ils posent le bol dans l'herbe.
+narrateur|Nina cueille une fraise haute.
+narrateur|Elle la laisse tomber dans le bol.
+narrateur|Le bol sonne un petit ding.
+enfant-m|Ding !
+narrateur|En ce moment, Victorino lève la main.
 narrateur|Une fraise rouge est trop haut.
-narrateur|Victorino lève la main.
-narrateur|Il n'arrive pas.
-enfant-m|Elle est trop haut.
-maman|Il y en a en bas aussi.
-narrateur|Nina cueille la haute.
-narrateur|Victorino cueille une basse.
-narrateur|La basse sent le sucre.
-enfant-m|Elle est chaude !
-maman|Le soleil l'a chauffée.
-maman|Vous jouez ensemble.
-maman|On peut jouer ensemble.
-narrateur|Le bol sonne un peu.
-narrateur|Deux fraises roulent dedans.
-copine|Encore une ?
-enfant-m|Oui.
+narrateur|Sa main n'arrive pas.
+enfant-m|Elle est trop haut !
+narrateur|Il saisit le bol trop vite.
+narrateur|Le bol penche vers l'herbe.
+narrateur|L'éclat d'émail saute près du bol.
+enfant-m|Oh.
+narrateur|Le sourire de Victorino disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+enfant-m|Ça ne veut pas !
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tes doigts sont près du bol ?
+enfant-m|Oui, papa.
+maman|On essuie tes genoux.
+maman|Voilà.
+enfant-m|C'est tiède.
+papa|C'est la terre, Victorino.
 narrateur|Une feuille colle au poignet.
-narrateur|Victorino la retire, tout doux.
-narrateur|La terre reste sur ses genoux.
-narrateur|Elle est chaude, un peu sèche.
-maman|On laisse l'abeille ?
-enfant-m|Oui.
-maman|Tu as de la terre aux genoux.
-enfant-m|C'est le jardin.</t>
+narrateur|Victorino la retire.
+narrateur|Nina reste près des hautes feuilles.
+narrateur|Elle ne dit rien.
+enfant-m|La haute, Nina !
+narrateur|Victorino veut la haute, tout de suite.
+narrateur|Il tend le bras trop loin.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>jardin,bol,feuilles</t>
         </is>
       </c>
     </row>
@@ -1407,12 +1433,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino invite Nina. Que font-ils ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino invite &lt;emphasis level="moderate"&gt;Nina&lt;/emphasis&gt;. Que font-ils ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nora invite Hugo. Que font-ils ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorino invite &lt;emphasis&gt;Nina&lt;/emphasis&gt;. Que font-ils ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1475,7 +1501,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1483,10 +1509,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1501,34 +1527,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1537,13 +1567,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1553,7 +1583,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_invite_nina_ils_restent_pres_des_fraisiers; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1586,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina pose une fraise haute. Victorino pose une fraise basse. Le bol se remplit. Le fond devient rouge. Il est lourd, maintenant. Oui. Petit ou grand, on cueille. Ils tapent des mains, tout doux. Une goutte de jus brille. Elle est sur le menton de Nina. C'est sucré. La mienne aussi. Vous avez des tailles différentes. Et vous jouez ensemble. Le bol est plein, non ? Oui, maman. Le plaid attend sous le cerisier. Il sent encore le linge. L'abeille s'éloigne. Les feuilles bougent un peu. On y va ? Oui.</t>
+          <t>Victorino veut la fraise haute. Il saute un peu. Sa main touche la feuille. La fraise reste trop haut. Je l'ai ! Nina avance la main aussi. Les deux mains se heurtent. La fraise bascule. Le bol tremble dans l'herbe. Oh. Non. Le sourire ne revient pas. Victorino refuse de foncer. Il repose le bol. Personne ne dit la suite. Il écoute les feuilles du jardin. Il regarde le bol, puis Nina. Sur le bord, l'éclat d'émail revient. Il est là. Une fraise basse touche son genou. Il la cueille près du genou. Il la fait rouler vers le bol. La fraise tombe dedans. Le bol sonne. Ding. Nina cueille une haute. Elle la laisse tomber. Le bol sonne, plus fort. Ding. La mienne aussi. Merci, Victorino. Papa a regardé jusqu'au bout. Le bol est lourd, non ? Oui, maman. On va sous le cerisier ? Le goûter, oui. Le ventre de Victorino se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina pose une fraise haute. Victorino pose une fraise basse. Le bol se remplit. Le fond devient rouge. Il est lourd, maintenant. Oui. Petit ou grand, on cueille. Ils tapent des mains, tout doux. Une goutte de jus brille. Elle est sur le menton de Nina. C'est sucré. La mienne aussi. Vous avez des tailles différentes. Et vous jouez ensemble. Le bol est plein, non ? Oui, maman. Le plaid attend sous le cerisier. Il sent encore le linge. L'abeille s'éloigne. Les feuilles bougent un peu. On y va ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino veut la fraise haute. Il saute un peu. Sa main touche la feuille. La fraise reste trop haut. Je l'ai ! Nina avance la main aussi. Les deux mains se heurtent. La fraise bascule. Le bol tremble dans l'herbe. Oh. Non. Le sourire ne revient pas. Victorino refuse de foncer. Il repose le bol. Personne ne dit la suite. Il écoute les feuilles du jardin. Il regarde le bol, puis Nina. Sur le bord, l'éclat d'émail revient. Il est là. Une fraise basse touche son genou. Il la cueille près du genou. Il la fait rouler vers le bol. La fraise tombe dedans. Le bol sonne. &lt;emphasis level="moderate"&gt;Ding&lt;/emphasis&gt;. Nina cueille une haute. Elle la laisse tomber. Le bol sonne, plus fort. Ding. La mienne aussi. Merci, Victorino. Papa a regardé jusqu'au bout. Le bol est lourd, non ? Oui, maman. On va sous le cerisier ? Le goûter, oui. Le ventre de Victorino se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nora a invité. Hugo a dit oui. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Ils jouent ensemble.&lt;/slow&gt; [pause]</t>
+          <t>Victorino veut la fraise haute. Il saute un peu. Sa main touche la feuille. La fraise reste trop haut. Je l'ai ! Nina avance la main aussi. Les deux mains se heurtent. La fraise bascule. Le bol tremble dans l'herbe. Oh. Non. Le sourire ne revient pas. Victorino refuse de foncer. Il repose le bol. Personne ne dit la suite. Il écoute les feuilles du jardin. Il regarde le bol, puis Nina. Sur le bord, l'éclat d'émail revient. Il est là. Une fraise basse touche son genou. Il la cueille près du genou. Il la fait rouler vers le bol. La fraise tombe dedans. Le bol sonne. &lt;emphasis&gt;Ding&lt;/emphasis&gt;. Nina cueille une haute. Elle la laisse tomber. Le bol sonne, plus fort. Ding. La mienne aussi. Merci, Victorino. Papa a regardé jusqu'au bout. Le bol est lourd, non ? Oui, maman. On va sous le cerisier ? Le goûter, oui. Le ventre de Victorino se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,18 +1673,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1677,30 +1707,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>Ding</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1739,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,37 +1751,57 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_cueille_bas_nina_haut; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina pose une fraise haute.
-narrateur|Victorino pose une fraise basse.
-narrateur|Le bol se remplit.
-narrateur|Le fond devient rouge.
-enfant-m|Il est lourd, maintenant.
-maman|Oui.
-maman|Petit ou grand, on cueille.
-narrateur|Ils tapent des mains, tout doux.
-narrateur|Une goutte de jus brille.
-narrateur|Elle est sur le menton de Nina.
-copine|C'est sucré.
+          <t>narrateur|Victorino veut la fraise haute.
+narrateur|Il saute un peu.
+narrateur|Sa main touche la feuille.
+narrateur|La fraise reste trop haut.
+enfant-m|Je l'ai !
+narrateur|Nina avance la main aussi.
+narrateur|Les deux mains se heurtent.
+narrateur|La fraise bascule.
+narrateur|Le bol tremble dans l'herbe.
+enfant-m|Oh.
+copine|Non.
+narrateur|Le sourire ne revient pas.
+narrateur|Victorino refuse de foncer.
+narrateur|Il repose le bol.
+narrateur|Personne ne dit la suite.
+narrateur|Il écoute les feuilles du jardin.
+narrateur|Il regarde le bol, puis Nina.
+narrateur|Sur le bord, l'éclat d'émail revient.
+enfant-m|Il est là.
+narrateur|Une fraise basse touche son genou.
+narrateur|Il la cueille près du genou.
+narrateur|Il la fait rouler vers le bol.
+narrateur|La fraise tombe dedans.
+narrateur|Le bol sonne.
+enfant-m|Ding.
+narrateur|Nina cueille une haute.
+narrateur|Elle la laisse tomber.
+narrateur|Le bol sonne, plus fort.
+copine|Ding.
 enfant-m|La mienne aussi.
-maman|Vous avez des tailles différentes.
-maman|Et vous jouez ensemble.
-maman|Le bol est plein, non ?
+papa|Merci, Victorino.
+narrateur|Papa a regardé jusqu'au bout.
+maman|Le bol est lourd, non ?
 enfant-m|Oui, maman.
-narrateur|Le plaid attend sous le cerisier.
-narrateur|Il sent encore le linge.
-narrateur|L'abeille s'éloigne.
-narrateur|Les feuilles bougent un peu.
-enfant-m|On y va ?
-copine|Oui.</t>
+papa|On va sous le cerisier ?
+enfant-m|Le goûter, oui.
+narrateur|Le ventre de Victorino se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>bol,fraises</t>
         </is>
       </c>
     </row>
@@ -1778,17 +1828,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On pose le bol sur le plaid ? Oui. Victorino pose le bol. Nina pose le panier. Les fraises sentent fort. Tu as fini de poser le bol ? Oui, maman. Ils s'assoient sur le plaid. Le plaid est un peu rêche. À demain. À demain. Le jardin redevient calme. Le bol émaillé n'est plus froid.</t>
+          <t>Ils marchent vers le plaid. L'ombre du cerisier est fraîche. Les fraises sentent fort. Je le porte ! Victorino lève le bol trop haut. Ses bras tremblent un peu. Une fraise roule vers l'herbe. Ça roule ! Nina veut le reprendre, d'un coup. Le bol penche de l'autre côté. Oh. Victorino refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde le bol. Il écoute le cerisier. En bas, moi. Nina ne dit rien. Elle prend le bord, plus haut. Victorino tient le fond. Le bol ne penche plus. Il est lourd. Oui. Tes pieds sont dans l'herbe ? Oui, papa. On pose le bol ? Sur le plaid. Ils posent le bol sur le plaid. Le plaid est un peu rêche. Victorino s'assoit près du bol. Nina s'assoit, les genoux plus hauts. Une basse ! Il fait rouler une fraise. Elle tombe dans le bol. Nina en laisse tomber une. Le bol sonne deux fois. Ding ding. Tu l'entends, le petit bruit ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On pose le bol sur le plaid ? Oui. Victorino pose le bol. Nina pose le panier. Les fraises sentent fort. Tu as fini de poser le bol ? Oui, maman. Ils s'assoient sur le plaid. Le plaid est un peu rêche. À demain. À demain. Le jardin redevient calme. Le bol émaillé n'est plus froid.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils marchent vers le plaid. L'ombre du cerisier est fraîche. Les fraises sentent fort. Je le porte ! Victorino lève le &lt;emphasis level="moderate"&gt;bol&lt;/emphasis&gt; trop haut. Ses bras tremblent un peu. Une fraise roule vers l'herbe. Ça roule ! Nina veut le reprendre, d'un coup. Le bol penche de l'autre côté. Oh. Victorino refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde le bol. Il écoute le cerisier. En bas, moi. Nina ne dit rien. Elle prend le bord, plus haut. Victorino tient le fond. Le bol ne penche plus. Il est lourd. Oui. Tes pieds sont dans l'herbe ? Oui, papa. On pose le bol ? Sur le plaid. Ils posent le bol sur le plaid. Le plaid est un peu rêche. Victorino s'assoit près du bol. Nina s'assoit, les genoux plus hauts. Une basse ! Il fait rouler une fraise. Elle tombe dans le bol. Nina en laisse tomber une. Le bol sonne deux fois. Ding ding. Tu l'entends, le petit bruit ? Oui, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le soleil baisse un peu. Maman dit : on range. Nora range un seau. Hugo range une pelle. Ils se disent à de&lt;emphasis&gt;main&lt;/emphasis&gt;.&lt;/slow&gt; [pause]</t>
+          <t>Ils marchent vers le plaid. L'ombre du cerisier est fraîche. Les fraises sentent fort. Je le porte ! Victorino lève le &lt;emphasis&gt;bol&lt;/emphasis&gt; trop haut. Ses bras tremblent un peu. Une fraise roule vers l'herbe. Ça roule ! Nina veut le reprendre, d'un coup. Le bol penche de l'autre côté. Oh. Victorino refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde le bol. Il écoute le cerisier. En bas, moi. Nina ne dit rien. Elle prend le bord, plus haut. Victorino tient le fond. Le bol ne penche plus. Il est lourd. Oui. Tes pieds sont dans l'herbe ? Oui, papa. On pose le bol ? Sur le plaid. Ils posent le bol sur le plaid. Le plaid est un peu rêche. Victorino s'assoit près du bol. Nina s'assoit, les genoux plus hauts. Une basse ! Il fait rouler une fraise. Elle tombe dans le bol. Nina en laisse tomber une. Le bol sonne deux fois. Ding ding. Tu l'entends, le petit bruit ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1835,18 +1885,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1869,30 +1919,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>bol</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1901,10 +1951,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1913,24 +1963,60 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_tient_le_fond_nina_le_bord; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On pose le bol sur le plaid ?
-enfant-m|Oui.
-narrateur|Victorino pose le bol.
-narrateur|Nina pose le panier.
+          <t>narrateur|Ils marchent vers le plaid.
+narrateur|L'ombre du cerisier est fraîche.
 narrateur|Les fraises sentent fort.
-maman|Tu as fini de poser le bol ?
-enfant-m|Oui, maman.
-narrateur|Ils s'assoient sur le plaid.
+enfant-m|Je le porte !
+narrateur|Victorino lève le bol trop haut.
+narrateur|Ses bras tremblent un peu.
+narrateur|Une fraise roule vers l'herbe.
+enfant-m|Ça roule !
+narrateur|Nina veut le reprendre, d'un coup.
+narrateur|Le bol penche de l'autre côté.
+enfant-m|Oh.
+narrateur|Victorino refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Il regarde le bol.
+narrateur|Il écoute le cerisier.
+enfant-m|En bas, moi.
+narrateur|Nina ne dit rien.
+narrateur|Elle prend le bord, plus haut.
+narrateur|Victorino tient le fond.
+narrateur|Le bol ne penche plus.
+enfant-m|Il est lourd.
+copine|Oui.
+papa|Tes pieds sont dans l'herbe ?
+enfant-m|Oui, papa.
+maman|On pose le bol ?
+enfant-m|Sur le plaid.
+narrateur|Ils posent le bol sur le plaid.
 narrateur|Le plaid est un peu rêche.
-copine|À demain.
-enfant-m|À demain.
-narrateur|Le jardin redevient calme.
-narrateur|Le bol émaillé n'est plus froid.</t>
+narrateur|Victorino s'assoit près du bol.
+narrateur|Nina s'assoit, les genoux plus hauts.
+enfant-m|Une basse !
+narrateur|Il fait rouler une fraise.
+narrateur|Elle tombe dans le bol.
+narrateur|Nina en laisse tomber une.
+narrateur|Le bol sonne deux fois.
+enfant-m|Ding ding.
+papa|Tu l'entends, le petit bruit ?
+enfant-m|Oui, papa.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>plaid,pas</t>
         </is>
       </c>
     </row>
@@ -1957,17 +2043,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>On a un bol de fraises. On a cueilli ensemble. Bravo, Victorino. Une goutte sèche sur le bord.</t>
+          <t>Ils restent sur le plaid. Le bol n'est plus froid. Comme tout à l'heure, papa ! Tu le vois, le petit bord ? Oui, l'éclat. On est bien, ici. Le cerisier sent un peu le sucre. Victorino glisse le pied, sans se presser. On le sent, maman. Tu le sens sur tes joues ? Oui, il est tiède. Une goutte de jus sèche au bord. L'éclat, il est là. On le laisse ? Oui. L'éclat d'émail tient sur le bol.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>On a un bol de fraises. On a cueilli ensemble. Bravo, Victorino. Une goutte sèche sur le bord.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent sur le plaid. Le bol n'est plus froid. Comme tout à l'heure, papa ! Tu le vois, le petit bord ? Oui, l'éclat. On est bien, ici. Le cerisier sent un peu le sucre. Victorino glisse le pied, sans se presser. On le sent, maman. Tu le sens sur tes joues ? Oui, il est tiède. Une goutte de jus sèche au bord. L'éclat, il est là. On le laisse ? Oui. L'&lt;emphasis level="moderate"&gt;éclat d'émail&lt;/emphasis&gt; tient sur le bol.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent sur le plaid. Le bol n'est plus froid. Comme tout à l'heure, papa ! Tu le vois, le petit bord ? Oui, l'éclat. On est bien, ici. Le cerisier sent un peu le sucre. Victorino glisse le pied, sans se presser. On le sent, maman. Tu le sens sur tes joues ? Oui, il est tiède. Une goutte de jus sèche au bord. L'éclat, il est là. On le laisse ? Oui. L'&lt;emphasis&gt;éclat d'émail&lt;/emphasis&gt; tient sur le bol.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2014,7 +2100,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2022,7 +2108,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2034,12 +2120,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2048,17 +2134,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'émail</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2067,11 +2157,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2080,27 +2170,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bol; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|On a un bol de fraises.
-enfant-m|On a cueilli ensemble.
-maman|Bravo, Victorino.
-narrateur|Une goutte sèche sur le bord.</t>
+          <t>narrateur|Ils restent sur le plaid.
+narrateur|Le bol n'est plus froid.
+enfant-m|Comme tout à l'heure, papa !
+papa|Tu le vois, le petit bord ?
+enfant-m|Oui, l'éclat.
+maman|On est bien, ici.
+narrateur|Le cerisier sent un peu le sucre.
+narrateur|Victorino glisse le pied, sans se presser.
+enfant-m|On le sent, maman.
+maman|Tu le sens sur tes joues ?
+enfant-m|Oui, il est tiède.
+narrateur|Une goutte de jus sèche au bord.
+enfant-m|L'éclat, il est là.
+papa|On le laisse ?
+enfant-m|Oui.
+narrateur|L'éclat d'émail tient sur le bol.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>cerisier,bol</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2199,6 +2310,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>